<commit_message>
corectare suprascriere db cu date vechi peste cele noi, corectare cale semnatura tehnician 2
</commit_message>
<xml_diff>
--- a/dist/Gestiune_clienti_sqlite_portabil_v4/_internal/mapping_tehnician.xlsx
+++ b/dist/Gestiune_clienti_sqlite_portabil_v4/_internal/mapping_tehnician.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gestionare_clienti_cu SQLite\pythonProject1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5965E363-BA63-419B-BD9D-9EE34C9799FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF0D3B3-DD8F-4A74-A037-A1211A217907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,10 +51,10 @@
     <t>Semnatura</t>
   </si>
   <si>
-    <t>grecu.png</t>
-  </si>
-  <si>
     <t>semnaturi/pop.png</t>
+  </si>
+  <si>
+    <t>semnaturi/grecu.png</t>
   </si>
 </sst>
 </file>
@@ -405,7 +405,7 @@
         <v>236</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -419,7 +419,7 @@
         <v>1817</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>